<commit_message>
Fixes component list match (we have perfect match)
</commit_message>
<xml_diff>
--- a/sch/components.xlsx
+++ b/sch/components.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\miha\Desktop\vezje-idp\kicad\sch\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66667DF9-155D-4464-A506-328CD4800B07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F7835F9-2275-499B-89E0-5C8DAB8BD279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" xr2:uid="{6172FD7F-16CD-47D1-A3E4-D63AC8EC044E}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="929" uniqueCount="428">
   <si>
     <t>ID</t>
   </si>
@@ -1086,9 +1086,6 @@
     <t>S14</t>
   </si>
   <si>
-    <t>C74</t>
-  </si>
-  <si>
     <t>S367</t>
   </si>
   <si>
@@ -1125,9 +1122,6 @@
     <t>33R</t>
   </si>
   <si>
-    <t>LS74</t>
-  </si>
-  <si>
     <t>MC14411</t>
   </si>
   <si>
@@ -1146,24 +1140,12 @@
     <t>4K7</t>
   </si>
   <si>
-    <t>P4?</t>
-  </si>
-  <si>
-    <t>P2?</t>
-  </si>
-  <si>
     <t>P1</t>
   </si>
   <si>
     <t>4.7K</t>
   </si>
   <si>
-    <t>4K7?</t>
-  </si>
-  <si>
-    <t>Z80CTC</t>
-  </si>
-  <si>
     <t>S20</t>
   </si>
   <si>
@@ -1215,9 +1197,6 @@
     <t>S38</t>
   </si>
   <si>
-    <t>S629?</t>
-  </si>
-  <si>
     <t>S393</t>
   </si>
   <si>
@@ -1260,9 +1239,6 @@
     <t>Z80 PIO (MK 3881)</t>
   </si>
   <si>
-    <t>P3 / S04</t>
-  </si>
-  <si>
     <t>2n 2 (?)</t>
   </si>
   <si>
@@ -1300,6 +1276,39 @@
   </si>
   <si>
     <t>390pF</t>
+  </si>
+  <si>
+    <t>P3</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>P4</t>
+  </si>
+  <si>
+    <t>S629</t>
+  </si>
+  <si>
+    <t>Z80 CTC</t>
+  </si>
+  <si>
+    <t>LS74 / S74</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Read as black-brown-red. Most likely it is green-brown-red (5K1).</t>
+  </si>
+  <si>
+    <t>"E75" (pg. 7)</t>
+  </si>
+  <si>
+    <t>Value Ref3</t>
+  </si>
+  <si>
+    <t>MM2716Q (EPROM)</t>
   </si>
 </sst>
 </file>
@@ -1354,11 +1363,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1673,15 +1682,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A507EC0B-FECA-46C5-861D-53A4B99CDA9D}">
-  <dimension ref="A1:G283"/>
+  <dimension ref="A1:I283"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="3" max="3" width="15.83984375" customWidth="1"/>
     <col min="4" max="4" width="15.5234375" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.20703125" customWidth="1"/>
+    <col min="7" max="7" width="31.3125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.15625" customWidth="1"/>
+    <col min="9" max="9" width="53.9453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>343</v>
       </c>
@@ -1703,8 +1714,14 @@
       <c r="G1" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="H1" t="s">
+        <v>426</v>
+      </c>
+      <c r="I1" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2">
         <v>79</v>
       </c>
@@ -1715,7 +1732,7 @@
         <v>77</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -1724,11 +1741,11 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A3">
         <v>71</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E3">
@@ -1738,7 +1755,7 @@
         <v>1.6</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4">
         <v>96</v>
       </c>
@@ -1755,7 +1772,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A5">
         <v>104</v>
       </c>
@@ -1772,7 +1789,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A6">
         <v>199</v>
       </c>
@@ -1789,7 +1806,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A7">
         <v>121</v>
       </c>
@@ -1800,7 +1817,7 @@
         <v>118</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>412</v>
+        <v>404</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -1809,7 +1826,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A8">
         <v>75</v>
       </c>
@@ -1820,7 +1837,7 @@
         <v>73</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>424</v>
+        <v>416</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -1829,7 +1846,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A9">
         <v>97</v>
       </c>
@@ -1846,7 +1863,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A10">
         <v>83</v>
       </c>
@@ -1857,7 +1874,7 @@
         <v>81</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>413</v>
+        <v>405</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -1866,7 +1883,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A11">
         <v>98</v>
       </c>
@@ -1883,7 +1900,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A12">
         <v>99</v>
       </c>
@@ -1900,7 +1917,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A13">
         <v>100</v>
       </c>
@@ -1917,7 +1934,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A14">
         <v>101</v>
       </c>
@@ -1934,7 +1951,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A15">
         <v>102</v>
       </c>
@@ -1951,7 +1968,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A16">
         <v>174</v>
       </c>
@@ -1962,7 +1979,7 @@
         <v>168</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>414</v>
+        <v>406</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -1982,7 +1999,7 @@
         <v>169</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>415</v>
+        <v>407</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2012,7 +2029,7 @@
       <c r="A19">
         <v>72</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>71</v>
       </c>
       <c r="E19">
@@ -2033,7 +2050,7 @@
         <v>239</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>416</v>
+        <v>408</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -2053,7 +2070,7 @@
         <v>12</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>417</v>
+        <v>409</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -2076,7 +2093,7 @@
         <v>13</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>417</v>
+        <v>409</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -2092,7 +2109,7 @@
       <c r="A23">
         <v>61</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E23">
@@ -2113,7 +2130,7 @@
         <v>10</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>418</v>
+        <v>410</v>
       </c>
       <c r="E24">
         <v>1</v>
@@ -2136,7 +2153,7 @@
         <v>242</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>419</v>
+        <v>411</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -2149,7 +2166,7 @@
       <c r="A26">
         <v>62</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="3" t="s">
         <v>60</v>
       </c>
       <c r="E26">
@@ -2170,7 +2187,7 @@
         <v>51</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>420</v>
+        <v>412</v>
       </c>
       <c r="E27">
         <v>1</v>
@@ -2190,7 +2207,7 @@
         <v>40</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>420</v>
+        <v>412</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2210,7 +2227,7 @@
         <v>38</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>421</v>
+        <v>413</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2230,7 +2247,7 @@
         <v>39</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>416</v>
+        <v>408</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -2260,7 +2277,7 @@
       <c r="A32">
         <v>1</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E32">
@@ -2277,7 +2294,7 @@
       <c r="A33">
         <v>15</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E33">
@@ -2294,7 +2311,7 @@
       <c r="A34">
         <v>24</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E34">
@@ -2311,7 +2328,7 @@
       <c r="A35">
         <v>48</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E35">
@@ -2328,7 +2345,7 @@
       <c r="A36">
         <v>74</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E36">
@@ -2345,7 +2362,7 @@
       <c r="A37">
         <v>108</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E37">
@@ -2362,7 +2379,7 @@
       <c r="A38">
         <v>125</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B38" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E38">
@@ -2379,7 +2396,7 @@
       <c r="A39">
         <v>130</v>
       </c>
-      <c r="B39" s="4" t="s">
+      <c r="B39" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E39">
@@ -2396,7 +2413,7 @@
       <c r="A40">
         <v>144</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="B40" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E40">
@@ -2413,7 +2430,7 @@
       <c r="A41">
         <v>163</v>
       </c>
-      <c r="B41" s="4" t="s">
+      <c r="B41" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E41">
@@ -2430,7 +2447,7 @@
       <c r="A42">
         <v>186</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="B42" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E42">
@@ -2447,7 +2464,7 @@
       <c r="A43">
         <v>195</v>
       </c>
-      <c r="B43" s="4" t="s">
+      <c r="B43" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E43">
@@ -2464,7 +2481,7 @@
       <c r="A44">
         <v>213</v>
       </c>
-      <c r="B44" s="4" t="s">
+      <c r="B44" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E44">
@@ -2481,7 +2498,7 @@
       <c r="A45">
         <v>221</v>
       </c>
-      <c r="B45" s="4" t="s">
+      <c r="B45" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E45">
@@ -2498,7 +2515,7 @@
       <c r="A46">
         <v>248</v>
       </c>
-      <c r="B46" s="4" t="s">
+      <c r="B46" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E46">
@@ -2515,7 +2532,7 @@
       <c r="A47">
         <v>264</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="B47" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E47">
@@ -2562,7 +2579,7 @@
         <v>6</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="E49">
         <v>1</v>
@@ -2631,7 +2648,7 @@
         <v>254</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="E52">
         <v>1</v>
@@ -2654,7 +2671,7 @@
         <v>247</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E53">
         <v>1</v>
@@ -2677,7 +2694,7 @@
         <v>248</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E54">
         <v>1</v>
@@ -2700,7 +2717,7 @@
         <v>249</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
       <c r="E55">
         <v>1</v>
@@ -2723,7 +2740,7 @@
         <v>250</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E56">
         <v>1</v>
@@ -2746,7 +2763,7 @@
         <v>251</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E57">
         <v>1</v>
@@ -2769,7 +2786,7 @@
         <v>252</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -2792,7 +2809,7 @@
         <v>7</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -2815,7 +2832,7 @@
         <v>57</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -2838,7 +2855,7 @@
         <v>58</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E61">
         <v>1</v>
@@ -2861,7 +2878,7 @@
         <v>49</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E62">
         <v>1</v>
@@ -2884,7 +2901,7 @@
         <v>48</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E63">
         <v>1</v>
@@ -2907,7 +2924,7 @@
         <v>29</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E64">
         <v>1</v>
@@ -2930,7 +2947,7 @@
         <v>30</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E65">
         <v>1</v>
@@ -2953,7 +2970,7 @@
         <v>31</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E66">
         <v>1</v>
@@ -2976,7 +2993,7 @@
         <v>22</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E67">
         <v>1</v>
@@ -3022,7 +3039,7 @@
         <v>23</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E69">
         <v>1</v>
@@ -3045,7 +3062,7 @@
         <v>24</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E70">
         <v>1</v>
@@ -3068,7 +3085,7 @@
         <v>8</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E71">
         <v>1</v>
@@ -3091,7 +3108,7 @@
         <v>9</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E72">
         <v>1</v>
@@ -3114,7 +3131,7 @@
         <v>15</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E73">
         <v>1</v>
@@ -3137,7 +3154,7 @@
         <v>16</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E74">
         <v>1</v>
@@ -3160,7 +3177,7 @@
         <v>120</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
       <c r="E75">
         <v>1</v>
@@ -3183,7 +3200,7 @@
         <v>121</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
       <c r="E76">
         <v>1</v>
@@ -3206,7 +3223,7 @@
         <v>119</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
       <c r="E77">
         <v>1</v>
@@ -3229,7 +3246,7 @@
         <v>110</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E78">
         <v>1</v>
@@ -3251,8 +3268,8 @@
       <c r="C79" t="s">
         <v>41</v>
       </c>
-      <c r="D79" s="3" t="s">
-        <v>353</v>
+      <c r="D79" s="2" t="s">
+        <v>360</v>
       </c>
       <c r="E79">
         <v>1</v>
@@ -3275,7 +3292,7 @@
         <v>106</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="E80">
         <v>1</v>
@@ -3298,7 +3315,7 @@
         <v>107</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="E81">
         <v>1</v>
@@ -3321,7 +3338,7 @@
         <v>108</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="E82">
         <v>1</v>
@@ -3344,7 +3361,7 @@
         <v>109</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="E83">
         <v>1</v>
@@ -3367,7 +3384,7 @@
         <v>92</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E84">
         <v>1</v>
@@ -3390,7 +3407,7 @@
         <v>91</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="E85">
         <v>1</v>
@@ -3413,7 +3430,7 @@
         <v>74</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E86">
         <v>1</v>
@@ -3436,7 +3453,7 @@
         <v>101</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E87">
         <v>1</v>
@@ -3459,7 +3476,7 @@
         <v>75</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -3482,7 +3499,7 @@
         <v>82</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E89">
         <v>1</v>
@@ -3528,7 +3545,7 @@
         <v>80</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>422</v>
+        <v>414</v>
       </c>
       <c r="E91">
         <v>1</v>
@@ -3551,7 +3568,7 @@
         <v>76</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E92">
         <v>1</v>
@@ -3652,7 +3669,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A97">
         <v>136</v>
       </c>
@@ -3663,7 +3680,7 @@
         <v>132</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E97">
         <v>1</v>
@@ -3675,7 +3692,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A98">
         <v>137</v>
       </c>
@@ -3686,7 +3703,7 @@
         <v>133</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E98">
         <v>1</v>
@@ -3698,7 +3715,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A99">
         <v>129</v>
       </c>
@@ -3709,7 +3726,7 @@
         <v>126</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>406</v>
+        <v>399</v>
       </c>
       <c r="E99">
         <v>1</v>
@@ -3721,7 +3738,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A100">
         <v>126</v>
       </c>
@@ -3732,7 +3749,7 @@
         <v>122</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>404</v>
+        <v>397</v>
       </c>
       <c r="E100">
         <v>1</v>
@@ -3744,7 +3761,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A101">
         <v>26</v>
       </c>
@@ -3755,7 +3772,7 @@
         <v>26</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E101">
         <v>1</v>
@@ -3767,7 +3784,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A102">
         <v>127</v>
       </c>
@@ -3777,7 +3794,7 @@
       <c r="C102" t="s">
         <v>123</v>
       </c>
-      <c r="D102" s="2">
+      <c r="D102" s="5">
         <v>2716</v>
       </c>
       <c r="E102">
@@ -3790,7 +3807,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A103">
         <v>128</v>
       </c>
@@ -3800,7 +3817,7 @@
       <c r="C103" t="s">
         <v>124</v>
       </c>
-      <c r="D103" s="2">
+      <c r="D103" s="5">
         <v>2716</v>
       </c>
       <c r="E103">
@@ -3810,10 +3827,13 @@
         <v>3.1</v>
       </c>
       <c r="G103" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>279</v>
+      </c>
+      <c r="H103" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A104">
         <v>141</v>
       </c>
@@ -3836,7 +3856,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A105">
         <v>134</v>
       </c>
@@ -3859,7 +3879,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A106">
         <v>133</v>
       </c>
@@ -3870,7 +3890,7 @@
         <v>129</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E106">
         <v>1</v>
@@ -3882,7 +3902,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A107">
         <v>132</v>
       </c>
@@ -3893,7 +3913,7 @@
         <v>128</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
       <c r="E107">
         <v>1</v>
@@ -3905,7 +3925,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A108">
         <v>131</v>
       </c>
@@ -3928,7 +3948,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A109">
         <v>172</v>
       </c>
@@ -3939,7 +3959,7 @@
         <v>166</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="E109">
         <v>1</v>
@@ -3951,7 +3971,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A110">
         <v>173</v>
       </c>
@@ -3974,7 +3994,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A111">
         <v>145</v>
       </c>
@@ -3997,7 +4017,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A112">
         <v>27</v>
       </c>
@@ -4008,7 +4028,7 @@
         <v>27</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E112">
         <v>1</v>
@@ -4100,7 +4120,7 @@
         <v>177</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>410</v>
+        <v>403</v>
       </c>
       <c r="E116">
         <v>1</v>
@@ -4123,7 +4143,7 @@
         <v>175</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="E117">
         <v>1</v>
@@ -4146,7 +4166,7 @@
         <v>161</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
       <c r="E118">
         <v>1</v>
@@ -4169,7 +4189,7 @@
         <v>162</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E119">
         <v>1</v>
@@ -4192,7 +4212,7 @@
         <v>163</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>378</v>
+        <v>421</v>
       </c>
       <c r="E120">
         <v>1</v>
@@ -4215,7 +4235,7 @@
         <v>164</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E121">
         <v>1</v>
@@ -4238,7 +4258,7 @@
         <v>165</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E122">
         <v>1</v>
@@ -4261,7 +4281,7 @@
         <v>17</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E123">
         <v>1</v>
@@ -4284,7 +4304,7 @@
         <v>171</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>396</v>
+        <v>420</v>
       </c>
       <c r="E124">
         <v>1</v>
@@ -4399,7 +4419,7 @@
         <v>218</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
       <c r="E129">
         <v>1</v>
@@ -4422,7 +4442,7 @@
         <v>215</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="E130">
         <v>1</v>
@@ -4445,7 +4465,7 @@
         <v>205</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E131">
         <v>1</v>
@@ -4468,7 +4488,7 @@
         <v>206</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>391</v>
+        <v>385</v>
       </c>
       <c r="E132">
         <v>1</v>
@@ -4491,7 +4511,7 @@
         <v>207</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="E133">
         <v>1</v>
@@ -4514,7 +4534,7 @@
         <v>18</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E134">
         <v>1</v>
@@ -4534,10 +4554,10 @@
         <v>208</v>
       </c>
       <c r="C135" t="s">
-        <v>201</v>
+        <v>425</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>394</v>
+        <v>355</v>
       </c>
       <c r="E135">
         <v>1</v>
@@ -4557,10 +4577,10 @@
         <v>201</v>
       </c>
       <c r="C136" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>356</v>
+        <v>388</v>
       </c>
       <c r="E136">
         <v>1</v>
@@ -4580,10 +4600,10 @@
         <v>199</v>
       </c>
       <c r="C137" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>366</v>
+        <v>355</v>
       </c>
       <c r="E137">
         <v>1</v>
@@ -4606,7 +4626,7 @@
         <v>193</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>361</v>
+        <v>422</v>
       </c>
       <c r="E138">
         <v>1</v>
@@ -4629,7 +4649,7 @@
         <v>203</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E139">
         <v>1</v>
@@ -4744,7 +4764,7 @@
         <v>219</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>373</v>
+        <v>419</v>
       </c>
       <c r="E144">
         <v>1</v>
@@ -4767,7 +4787,7 @@
         <v>19</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
       <c r="E145">
         <v>1</v>
@@ -4790,7 +4810,7 @@
         <v>216</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>374</v>
+        <v>418</v>
       </c>
       <c r="E146">
         <v>1</v>
@@ -4813,7 +4833,7 @@
         <v>209</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E147">
         <v>1</v>
@@ -4836,7 +4856,7 @@
         <v>210</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="E148">
         <v>1</v>
@@ -4859,7 +4879,7 @@
         <v>211</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="E149">
         <v>1</v>
@@ -4882,7 +4902,7 @@
         <v>202</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E150">
         <v>1</v>
@@ -4928,7 +4948,7 @@
         <v>197</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>397</v>
+        <v>390</v>
       </c>
       <c r="E152">
         <v>1</v>
@@ -4951,7 +4971,7 @@
         <v>194</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>398</v>
+        <v>391</v>
       </c>
       <c r="E153">
         <v>1</v>
@@ -5445,7 +5465,7 @@
         <v>62</v>
       </c>
       <c r="D181" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E181">
         <v>1</v>
@@ -5468,7 +5488,7 @@
         <v>50</v>
       </c>
       <c r="D182" s="2" t="s">
-        <v>403</v>
+        <v>396</v>
       </c>
       <c r="E182">
         <v>1</v>
@@ -5508,7 +5528,7 @@
         <v>47</v>
       </c>
       <c r="D184" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E184">
         <v>1</v>
@@ -5528,7 +5548,7 @@
         <v>46</v>
       </c>
       <c r="D185" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E185">
         <v>1</v>
@@ -5568,7 +5588,7 @@
         <v>44</v>
       </c>
       <c r="D187" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E187">
         <v>1</v>
@@ -5588,7 +5608,7 @@
         <v>43</v>
       </c>
       <c r="D188" s="2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E188">
         <v>1</v>
@@ -5631,7 +5651,7 @@
         <v>33</v>
       </c>
       <c r="D190" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E190">
         <v>1</v>
@@ -5677,7 +5697,7 @@
         <v>63</v>
       </c>
       <c r="D192" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E192">
         <v>1</v>
@@ -5723,7 +5743,7 @@
         <v>104</v>
       </c>
       <c r="D194" s="2" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="E194">
         <v>1</v>
@@ -5743,7 +5763,7 @@
         <v>105</v>
       </c>
       <c r="D195" s="2" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="E195">
         <v>1</v>
@@ -5763,7 +5783,7 @@
         <v>159</v>
       </c>
       <c r="D196" s="2" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="E196">
         <v>1</v>
@@ -5829,7 +5849,7 @@
         <v>21</v>
       </c>
       <c r="D199" s="2" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="E199">
         <v>1</v>
@@ -5852,7 +5872,7 @@
         <v>4</v>
       </c>
       <c r="D200" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E200">
         <v>1</v>
@@ -5872,10 +5892,10 @@
         <v>5</v>
       </c>
       <c r="C201" t="s">
-        <v>423</v>
+        <v>415</v>
       </c>
       <c r="D201" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E201">
         <v>1</v>
@@ -5898,7 +5918,7 @@
         <v>14</v>
       </c>
       <c r="D202" s="2" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="E202">
         <v>1</v>
@@ -5955,7 +5975,7 @@
         <v>64</v>
       </c>
       <c r="D205" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E205">
         <v>1</v>
@@ -6080,7 +6100,7 @@
         <v>103</v>
       </c>
       <c r="D212" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E212">
         <v>1</v>
@@ -6160,7 +6180,7 @@
         <v>65</v>
       </c>
       <c r="D216" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E216">
         <v>1</v>
@@ -6243,7 +6263,7 @@
         <v>148</v>
       </c>
       <c r="D220" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E220">
         <v>1</v>
@@ -6266,7 +6286,7 @@
         <v>149</v>
       </c>
       <c r="D221" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E221">
         <v>1</v>
@@ -6289,7 +6309,7 @@
         <v>150</v>
       </c>
       <c r="D222" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E222">
         <v>1</v>
@@ -6312,7 +6332,7 @@
         <v>151</v>
       </c>
       <c r="D223" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E223">
         <v>1</v>
@@ -6335,7 +6355,7 @@
         <v>152</v>
       </c>
       <c r="D224" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E224">
         <v>1</v>
@@ -6347,7 +6367,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="225" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A225">
         <v>158</v>
       </c>
@@ -6358,7 +6378,7 @@
         <v>153</v>
       </c>
       <c r="D225" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E225">
         <v>1</v>
@@ -6370,7 +6390,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="226" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="226" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A226">
         <v>159</v>
       </c>
@@ -6381,7 +6401,7 @@
         <v>154</v>
       </c>
       <c r="D226" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E226">
         <v>1</v>
@@ -6393,7 +6413,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="227" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="227" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A227">
         <v>67</v>
       </c>
@@ -6404,7 +6424,7 @@
         <v>66</v>
       </c>
       <c r="D227" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E227">
         <v>1</v>
@@ -6416,7 +6436,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="228" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A228">
         <v>160</v>
       </c>
@@ -6427,7 +6447,7 @@
         <v>155</v>
       </c>
       <c r="D228" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E228">
         <v>1</v>
@@ -6439,7 +6459,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="229" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="229" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A229">
         <v>161</v>
       </c>
@@ -6450,7 +6470,7 @@
         <v>156</v>
       </c>
       <c r="D229" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E229">
         <v>1</v>
@@ -6462,7 +6482,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="230" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A230">
         <v>162</v>
       </c>
@@ -6473,7 +6493,7 @@
         <v>157</v>
       </c>
       <c r="D230" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E230">
         <v>1</v>
@@ -6485,7 +6505,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="231" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A231">
         <v>176</v>
       </c>
@@ -6496,7 +6516,7 @@
         <v>170</v>
       </c>
       <c r="D231" s="2" t="s">
-        <v>402</v>
+        <v>395</v>
       </c>
       <c r="E231">
         <v>1</v>
@@ -6507,8 +6527,11 @@
       <c r="G231" t="s">
         <v>328</v>
       </c>
-    </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="I231" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="232" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A232">
         <v>196</v>
       </c>
@@ -6519,7 +6542,7 @@
         <v>188</v>
       </c>
       <c r="D232" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E232">
         <v>1</v>
@@ -6531,7 +6554,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="233" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="233" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A233">
         <v>200</v>
       </c>
@@ -6542,7 +6565,7 @@
         <v>192</v>
       </c>
       <c r="D233" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E233">
         <v>1</v>
@@ -6554,7 +6577,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="234" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A234">
         <v>204</v>
       </c>
@@ -6571,7 +6594,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="235" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A235">
         <v>207</v>
       </c>
@@ -6588,7 +6611,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="236" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="236" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A236">
         <v>178</v>
       </c>
@@ -6599,7 +6622,7 @@
         <v>172</v>
       </c>
       <c r="D236" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E236">
         <v>1</v>
@@ -6611,7 +6634,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="237" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="237" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A237">
         <v>179</v>
       </c>
@@ -6622,7 +6645,7 @@
         <v>173</v>
       </c>
       <c r="D237" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E237">
         <v>1</v>
@@ -6634,7 +6657,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="238" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="238" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A238">
         <v>230</v>
       </c>
@@ -6645,7 +6668,7 @@
         <v>220</v>
       </c>
       <c r="D238" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E238">
         <v>1</v>
@@ -6657,7 +6680,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="239" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A239">
         <v>231</v>
       </c>
@@ -6668,7 +6691,7 @@
         <v>221</v>
       </c>
       <c r="D239" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E239">
         <v>1</v>
@@ -6680,7 +6703,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="240" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="240" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A240">
         <v>232</v>
       </c>
@@ -6691,7 +6714,7 @@
         <v>222</v>
       </c>
       <c r="D240" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E240">
         <v>1</v>
@@ -6714,7 +6737,7 @@
         <v>223</v>
       </c>
       <c r="D241" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E241">
         <v>1</v>
@@ -6737,7 +6760,7 @@
         <v>224</v>
       </c>
       <c r="D242" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E242">
         <v>1</v>
@@ -6753,14 +6776,14 @@
       <c r="A243">
         <v>235</v>
       </c>
-      <c r="B243" s="5" t="s">
+      <c r="B243" s="4" t="s">
         <v>225</v>
       </c>
       <c r="C243" t="s">
         <v>225</v>
       </c>
       <c r="D243" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E243">
         <v>1</v>
@@ -6783,7 +6806,7 @@
         <v>226</v>
       </c>
       <c r="D244" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E244">
         <v>1</v>
@@ -6806,7 +6829,7 @@
         <v>227</v>
       </c>
       <c r="D245" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E245">
         <v>1</v>
@@ -6829,7 +6852,7 @@
         <v>228</v>
       </c>
       <c r="D246" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="E246">
         <v>1</v>
@@ -6852,7 +6875,7 @@
         <v>229</v>
       </c>
       <c r="D247" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="E247">
         <v>1</v>
@@ -6875,7 +6898,7 @@
         <v>67</v>
       </c>
       <c r="D248" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E248">
         <v>1</v>
@@ -6898,7 +6921,7 @@
         <v>230</v>
       </c>
       <c r="D249" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E249">
         <v>1</v>
@@ -6921,7 +6944,7 @@
         <v>231</v>
       </c>
       <c r="D250" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E250">
         <v>1</v>
@@ -6944,7 +6967,7 @@
         <v>232</v>
       </c>
       <c r="D251" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E251">
         <v>1</v>
@@ -6967,7 +6990,7 @@
         <v>233</v>
       </c>
       <c r="D252" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E252">
         <v>1</v>
@@ -6990,7 +7013,7 @@
         <v>234</v>
       </c>
       <c r="D253" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E253">
         <v>1</v>
@@ -7013,7 +7036,7 @@
         <v>235</v>
       </c>
       <c r="D254" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E254">
         <v>1</v>
@@ -7036,7 +7059,7 @@
         <v>236</v>
       </c>
       <c r="D255" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E255">
         <v>1</v>
@@ -7059,7 +7082,7 @@
         <v>237</v>
       </c>
       <c r="D256" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E256">
         <v>1</v>
@@ -7082,7 +7105,7 @@
         <v>256</v>
       </c>
       <c r="D257" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="E257">
         <v>1</v>
@@ -7105,7 +7128,7 @@
         <v>257</v>
       </c>
       <c r="D258" s="2" t="s">
-        <v>377</v>
+        <v>370</v>
       </c>
       <c r="E258">
         <v>1</v>
@@ -7128,7 +7151,7 @@
         <v>258</v>
       </c>
       <c r="D259" s="2" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="E259">
         <v>1</v>
@@ -7151,7 +7174,7 @@
         <v>259</v>
       </c>
       <c r="D260" s="2" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="E260">
         <v>1</v>
@@ -7174,7 +7197,7 @@
         <v>260</v>
       </c>
       <c r="D261" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E261">
         <v>1</v>
@@ -7197,7 +7220,7 @@
         <v>261</v>
       </c>
       <c r="D262" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="E262">
         <v>1</v>
@@ -7220,7 +7243,7 @@
         <v>262</v>
       </c>
       <c r="D263" s="2" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="E263">
         <v>1</v>
@@ -7243,7 +7266,7 @@
         <v>263</v>
       </c>
       <c r="D264" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E264">
         <v>1</v>
@@ -7266,7 +7289,7 @@
         <v>213</v>
       </c>
       <c r="D265" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="E265">
         <v>1</v>
@@ -7286,7 +7309,7 @@
         <v>240</v>
       </c>
       <c r="D266" s="2" t="s">
-        <v>399</v>
+        <v>392</v>
       </c>
       <c r="E266">
         <v>1</v>
@@ -7309,7 +7332,7 @@
         <v>241</v>
       </c>
       <c r="D267" s="2" t="s">
-        <v>399</v>
+        <v>392</v>
       </c>
       <c r="E267">
         <v>1</v>
@@ -7332,7 +7355,7 @@
         <v>243</v>
       </c>
       <c r="D268" s="2" t="s">
-        <v>401</v>
+        <v>394</v>
       </c>
       <c r="E268">
         <v>1</v>
@@ -7352,7 +7375,7 @@
         <v>68</v>
       </c>
       <c r="D269" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E269">
         <v>1</v>
@@ -7398,7 +7421,7 @@
         <v>217</v>
       </c>
       <c r="D271" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="E271">
         <v>1</v>
@@ -7421,7 +7444,7 @@
         <v>189</v>
       </c>
       <c r="D272" s="2" t="s">
-        <v>400</v>
+        <v>393</v>
       </c>
       <c r="E272">
         <v>1</v>
@@ -7444,7 +7467,7 @@
         <v>190</v>
       </c>
       <c r="D273" s="2" t="s">
-        <v>400</v>
+        <v>393</v>
       </c>
       <c r="E273">
         <v>1</v>
@@ -7550,7 +7573,7 @@
         <v>78</v>
       </c>
       <c r="D278" s="2" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="E278">
         <v>1</v>
@@ -7570,7 +7593,7 @@
         <v>79</v>
       </c>
       <c r="D279" s="2" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="E279">
         <v>1</v>
@@ -7631,7 +7654,7 @@
         <v>11</v>
       </c>
       <c r="D282" s="2" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="E282">
         <v>1</v>
@@ -7654,7 +7677,7 @@
         <v>158</v>
       </c>
       <c r="D283" s="2" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="E283">
         <v>1</v>

</xml_diff>